<commit_message>
new run results for cot prompting with tiny aya global model
</commit_message>
<xml_diff>
--- a/results/cot_inference/mgsm/tiny-aya-earth/summary_majority.xlsx
+++ b/results/cot_inference/mgsm/tiny-aya-earth/summary_majority.xlsx
@@ -460,14 +460,14 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>138</v>
+        <v>161</v>
       </c>
       <c r="D2" t="n">
         <v>250</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>55.2%</t>
+          <t>64.4%</t>
         </is>
       </c>
       <c r="F2" t="n">

</xml_diff>